<commit_message>
Document verified production environments
</commit_message>
<xml_diff>
--- a/results/submission/results.xlsx
+++ b/results/submission/results.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Submission" sheetId="1" r:id="Ra6072e9214c8472c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="2" r:id="R10cfe40218774d36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Submission" sheetId="1" r:id="R48bfd7245ca7415d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="2" r:id="Rc8a04cdda8654125"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -637,7 +637,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -648,7 +648,7 @@
         <x:color rgb="FF1D4ED8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
         </x:patternFill>
       </x:fill>
@@ -1210,7 +1210,7 @@
         <x:v>66.1</x:v>
       </x:c>
       <x:c r="AN2" s="34" t="str">
-        <x:v>BoltzGen 1 (boltzgen1_diverse.ckpt); BoltzIF (boltzgen1_ifold.ckpt); Boltz-2 (production package revision not archived)</x:v>
+        <x:v>BoltzGen/BoltzIF 0.2.0; Boltz-2 2.2.1 (production environment recovered 2026-08-15)</x:v>
       </x:c>
       <x:c r="AO2" s="34" t="str">
         <x:v>selected_for_synthesis</x:v>
@@ -1341,7 +1341,7 @@
         <x:v>79.5</x:v>
       </x:c>
       <x:c r="AN3" s="35" t="str">
-        <x:v>BoltzGen 1 (boltzgen1_diverse.ckpt); BoltzIF (boltzgen1_ifold.ckpt); Boltz-2 (production package revision not archived)</x:v>
+        <x:v>BoltzGen/BoltzIF 0.2.0; Boltz-2 2.2.1 (production environment recovered 2026-08-15)</x:v>
       </x:c>
       <x:c r="AO3" s="35" t="str">
         <x:v>selected_for_synthesis</x:v>
@@ -1472,7 +1472,7 @@
         <x:v>72.0</x:v>
       </x:c>
       <x:c r="AN4" s="35" t="str">
-        <x:v>BoltzGen 1 (boltzgen1_diverse.ckpt); BoltzIF (boltzgen1_ifold.ckpt); Boltz-2 (production package revision not archived)</x:v>
+        <x:v>BoltzGen/BoltzIF 0.2.0; Boltz-2 2.2.1 (production environment recovered 2026-08-15)</x:v>
       </x:c>
       <x:c r="AO4" s="35" t="str">
         <x:v>selected_for_synthesis</x:v>
@@ -1603,7 +1603,7 @@
         <x:v>79.3</x:v>
       </x:c>
       <x:c r="AN5" s="35" t="str">
-        <x:v>BoltzGen 1 (boltzgen1_diverse.ckpt); BoltzIF (boltzgen1_ifold.ckpt); Boltz-2 (production package revision not archived)</x:v>
+        <x:v>BoltzGen/BoltzIF 0.2.0; Boltz-2 2.2.1 (production environment recovered 2026-08-15)</x:v>
       </x:c>
       <x:c r="AO5" s="35" t="str">
         <x:v>selected_for_synthesis</x:v>
@@ -1734,7 +1734,7 @@
         <x:v>78.4</x:v>
       </x:c>
       <x:c r="AN6" s="35" t="str">
-        <x:v>BoltzGen 1 (boltzgen1_diverse.ckpt); BoltzIF (boltzgen1_ifold.ckpt); Boltz-2 (production package revision not archived)</x:v>
+        <x:v>BoltzGen/BoltzIF 0.2.0; Boltz-2 2.2.1 (production environment recovered 2026-08-15)</x:v>
       </x:c>
       <x:c r="AO6" s="35" t="str">
         <x:v>selected_for_synthesis</x:v>
@@ -1865,7 +1865,7 @@
         <x:v>72.8</x:v>
       </x:c>
       <x:c r="AN7" s="35" t="str">
-        <x:v>BoltzGen 1 (boltzgen1_diverse.ckpt); BoltzIF (boltzgen1_ifold.ckpt); Boltz-2 (production package revision not archived)</x:v>
+        <x:v>BoltzGen/BoltzIF 0.2.0; Boltz-2 2.2.1 (production environment recovered 2026-08-15)</x:v>
       </x:c>
       <x:c r="AO7" s="35" t="str">
         <x:v>selected_for_synthesis</x:v>
@@ -1996,7 +1996,7 @@
         <x:v>64.1</x:v>
       </x:c>
       <x:c r="AN8" s="35" t="str">
-        <x:v>BoltzGen 1 (boltzgen1_diverse.ckpt); BoltzIF (boltzgen1_ifold.ckpt); Boltz-2 (production package revision not archived)</x:v>
+        <x:v>BoltzGen/BoltzIF 0.2.0; Boltz-2 2.2.1 (production environment recovered 2026-08-15)</x:v>
       </x:c>
       <x:c r="AO8" s="35" t="str">
         <x:v>selected_for_synthesis</x:v>
@@ -2127,7 +2127,7 @@
         <x:v>72.9</x:v>
       </x:c>
       <x:c r="AN9" s="35" t="str">
-        <x:v>BoltzGen 1 (boltzgen1_diverse.ckpt); BoltzIF (boltzgen1_ifold.ckpt); Boltz-2 (production package revision not archived)</x:v>
+        <x:v>BoltzGen/BoltzIF 0.2.0; Boltz-2 2.2.1 (production environment recovered 2026-08-15)</x:v>
       </x:c>
       <x:c r="AO9" s="35" t="str">
         <x:v>selected_for_synthesis</x:v>
@@ -2258,7 +2258,7 @@
         <x:v>80.7</x:v>
       </x:c>
       <x:c r="AN10" s="35" t="str">
-        <x:v>BoltzGen 1 (boltzgen1_diverse.ckpt); BoltzIF (boltzgen1_ifold.ckpt); Boltz-2 (production package revision not archived)</x:v>
+        <x:v>BoltzGen/BoltzIF 0.2.0; Boltz-2 2.2.1 (production environment recovered 2026-08-15)</x:v>
       </x:c>
       <x:c r="AO10" s="35" t="str">
         <x:v>selected_for_synthesis</x:v>
@@ -2389,7 +2389,7 @@
         <x:v>64.7</x:v>
       </x:c>
       <x:c r="AN11" s="35" t="str">
-        <x:v>BoltzGen 1 (boltzgen1_diverse.ckpt); BoltzIF (boltzgen1_ifold.ckpt); Boltz-2 (production package revision not archived)</x:v>
+        <x:v>BoltzGen/BoltzIF 0.2.0; Boltz-2 2.2.1 (production environment recovered 2026-08-15)</x:v>
       </x:c>
       <x:c r="AO11" s="35" t="str">
         <x:v>selected_for_synthesis</x:v>
@@ -2520,7 +2520,7 @@
         <x:v>71.1</x:v>
       </x:c>
       <x:c r="AN12" s="35" t="str">
-        <x:v>BoltzGen 1 (boltzgen1_diverse.ckpt); BoltzIF (boltzgen1_ifold.ckpt); Boltz-2 (production package revision not archived)</x:v>
+        <x:v>BoltzGen/BoltzIF 0.2.0; Boltz-2 2.2.1 (production environment recovered 2026-08-15)</x:v>
       </x:c>
       <x:c r="AO12" s="35" t="str">
         <x:v>selected_for_synthesis</x:v>
@@ -2651,7 +2651,7 @@
         <x:v>67.2</x:v>
       </x:c>
       <x:c r="AN13" s="36" t="str">
-        <x:v>BoltzGen 1 (boltzgen1_diverse.ckpt); BoltzIF (boltzgen1_ifold.ckpt); Boltz-2 (production package revision not archived)</x:v>
+        <x:v>BoltzGen/BoltzIF 0.2.0; Boltz-2 2.2.1 (production environment recovered 2026-08-15)</x:v>
       </x:c>
       <x:c r="AO13" s="36" t="str">
         <x:v>selected_for_synthesis</x:v>
@@ -2670,7 +2670,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1791176b8a44d97"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50673e3da92f4071"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3192,7 +3192,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9de49e7f532a4e42"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4df0e5fc187440d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>